<commit_message>
7.1.6 played games history and history details
</commit_message>
<xml_diff>
--- a/process/resources/Pages.xlsx
+++ b/process/resources/Pages.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\Coding_WithGit\Vite-KingdomCreator-New\process\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C216BB-A15C-486F-867B-9CE5A5EDAE59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A7C6864-98A8-48E0-BFA2-2393DB03C247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1320" yWindow="1785" windowWidth="24975" windowHeight="13065" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pages" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7129" uniqueCount="5848">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7132" uniqueCount="5850">
   <si>
     <t>sep=</t>
   </si>
@@ -17891,6 +17891,12 @@
   </si>
   <si>
     <t>Jouer !</t>
+  </si>
+  <si>
+    <t>Unknown or invalid kingdom</t>
+  </si>
+  <si>
+    <t>Royaume inconnu ou invalide</t>
   </si>
 </sst>
 </file>
@@ -21948,7 +21954,15 @@
       <c r="A179" s="1" t="s">
         <v>5804</v>
       </c>
-      <c r="C179" s="33"/>
+      <c r="B179" s="25" t="s">
+        <v>5848</v>
+      </c>
+      <c r="C179" s="25" t="s">
+        <v>5848</v>
+      </c>
+      <c r="F179" t="s">
+        <v>5849</v>
+      </c>
       <c r="H179"/>
     </row>
     <row r="180" spans="1:9" ht="15" customHeight="1">

</xml_diff>